<commit_message>
IBWork Flow Automatd with no more range entry.  Will use trade flags in latesting earnings doc.
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28695" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="2" max="2"/>
@@ -440,14 +440,14 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Exit Type</t>
+          <t>IBKR Exit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>AEO</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -456,13 +456,18 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>112</v>
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -471,127 +476,32 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>GAP</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>VEEV</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>BJ</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>BURL</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>CIEN</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>VSCO</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>40</v>
+        <v>93</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed IB account to Algo account. Staged trades, updated Earning Doc
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="2" max="2"/>
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>CASY</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -456,7 +456,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -467,7 +467,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -487,18 +487,98 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>GAP</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>CTOS</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
           <t>long</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>93</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="C5" s="1" t="n">
+        <v>195</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>FERG</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>UNFI</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>WLFC</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>open</t>
         </is>

</xml_diff>

<commit_message>
Changes source of opening and closing prices from yfinance to IB Gateway.  Also changed some script names to be shorter.
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
@@ -472,7 +472,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
@@ -532,7 +532,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
@@ -552,7 +552,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
@@ -572,7 +572,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C8" s="1" t="n">

</xml_diff>

<commit_message>
Added Exit_IB_via_GW script which asks if I need to change any IB orders to MOC before sending orders
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,33 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading Algo/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_56BDF67C922DCD858E20AF4774604EA9598B8B36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02AD4D6-F0E8-4770-8852-857AD70C0173}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+  <si>
+    <t>Ticker</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Share Size</t>
+  </si>
+  <si>
+    <t>IBKR Exit</t>
+  </si>
+  <si>
+    <t>CASY</t>
+  </si>
+  <si>
+    <t>short</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>HPE</t>
+  </si>
+  <si>
+    <t>ORCL</t>
+  </si>
+  <si>
+    <t>CTOS</t>
+  </si>
+  <si>
+    <t>FERG</t>
+  </si>
+  <si>
+    <t>UNFI</t>
+  </si>
+  <si>
+    <t>WLFC</t>
+  </si>
+  <si>
+    <t>moc</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,84 +98,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -410,178 +407,124 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="11.28515625" customWidth="1" min="2" max="2"/>
-    <col width="12.7109375" customWidth="1" min="3" max="3"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>CASY</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>HPE</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
         <v>59</v>
       </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>CTOS</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
         <v>195</v>
       </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>FERG</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>UNFI</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
+      <c r="D5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
         <v>34</v>
       </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>WLFC</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
+      <c r="D7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1">
         <v>7</v>
       </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ToS exits, all MOC for a later script that will read that
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading Algo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_56BDF67C922DCD858E20AF4774604EA9598B8B36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02AD4D6-F0E8-4770-8852-857AD70C0173}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_56BDF67C922DCD250660FF925AE548FF598B89A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
   <si>
     <t>Ticker</t>
   </si>
@@ -34,6 +34,9 @@
     <t>IBKR Exit</t>
   </si>
   <si>
+    <t>ToS Exit</t>
+  </si>
+  <si>
     <t>CASY</t>
   </si>
   <si>
@@ -43,6 +46,9 @@
     <t>open</t>
   </si>
   <si>
+    <t>MOC</t>
+  </si>
+  <si>
     <t>HPE</t>
   </si>
   <si>
@@ -59,9 +65,6 @@
   </si>
   <si>
     <t>WLFC</t>
-  </si>
-  <si>
-    <t>moc</t>
   </si>
 </sst>
 </file>
@@ -117,10 +120,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -408,14 +407,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -428,103 +426,127 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1">
         <v>59</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
         <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1">
         <v>195</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1">
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Schwab API and authorized it.  Created a file to send live trades to ToS.
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,88 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading Algo/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_56BDF67C922DCD250660FF925AE548FF598B89A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" r:id="rId1"/>
+    <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
-  <si>
-    <t>Ticker</t>
-  </si>
-  <si>
-    <t>Direction</t>
-  </si>
-  <si>
-    <t>Share Size</t>
-  </si>
-  <si>
-    <t>IBKR Exit</t>
-  </si>
-  <si>
-    <t>ToS Exit</t>
-  </si>
-  <si>
-    <t>CASY</t>
-  </si>
-  <si>
-    <t>short</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>MOC</t>
-  </si>
-  <si>
-    <t>HPE</t>
-  </si>
-  <si>
-    <t>ORCL</t>
-  </si>
-  <si>
-    <t>CTOS</t>
-  </si>
-  <si>
-    <t>FERG</t>
-  </si>
-  <si>
-    <t>UNFI</t>
-  </si>
-  <si>
-    <t>WLFC</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -101,24 +46,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -406,147 +410,217 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+    <col width="12.42578125" customWidth="1" min="1" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>CASY</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>CTOS</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>207</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>FERG</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>UNFI</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>WLFC</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>59</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1">
-        <v>195</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="1">
-        <v>34</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>8</v>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added error handling when sending trades if there are none. This way the autoscheduler will know the script ran successfully and not get errors and try again
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" customWidth="1" min="1" max="5"/>
@@ -451,16 +451,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -468,156 +468,6 @@
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>HPE</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>59</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>CTOS</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>207</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>FERG</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>UNFI</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>WLFC</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
         </is>

</xml_diff>

<commit_message>
Removed some user prompts to further automate.
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" customWidth="1" min="1" max="5"/>
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>BMBL</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>49</v>
+        <v>445</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -468,6 +468,106 @@
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>PATH</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>DKS</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>OLLI</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
         </is>

</xml_diff>

<commit_message>
Removed space in Trading Algo folder, now Trading_Algo
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,33 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading Algo/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_56BD516C9400D595094DDB9E8A655EF7598B8449" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+  <si>
+    <t>Ticker</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Share Size</t>
+  </si>
+  <si>
+    <t>IBKR Exit</t>
+  </si>
+  <si>
+    <t>ToS Exit</t>
+  </si>
+  <si>
+    <t>BMBL</t>
+  </si>
+  <si>
+    <t>short</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>MOC</t>
+  </si>
+  <si>
+    <t>PATH</t>
+  </si>
+  <si>
+    <t>long</t>
+  </si>
+  <si>
+    <t>DG</t>
+  </si>
+  <si>
+    <t>DKS</t>
+  </si>
+  <si>
+    <t>OLLI</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,83 +98,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -410,167 +403,113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="12.42578125" customWidth="1" min="1" max="5"/>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>BMBL</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
         <v>445</v>
       </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>PATH</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1">
         <v>108</v>
       </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>DG</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1">
         <v>9</v>
       </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>DKS</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="C5" s="1">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>OLLI</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
         <v>12</v>
       </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change Stage Trades to take exit from Latest Earnings Doc
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,85 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading Algo/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_56BD516C9400D595094DDB9E8A655EF7598B8449" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" r:id="rId1"/>
+    <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
-  <si>
-    <t>Ticker</t>
-  </si>
-  <si>
-    <t>Direction</t>
-  </si>
-  <si>
-    <t>Share Size</t>
-  </si>
-  <si>
-    <t>IBKR Exit</t>
-  </si>
-  <si>
-    <t>ToS Exit</t>
-  </si>
-  <si>
-    <t>BMBL</t>
-  </si>
-  <si>
-    <t>short</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>MOC</t>
-  </si>
-  <si>
-    <t>PATH</t>
-  </si>
-  <si>
-    <t>long</t>
-  </si>
-  <si>
-    <t>DG</t>
-  </si>
-  <si>
-    <t>DKS</t>
-  </si>
-  <si>
-    <t>OLLI</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -98,24 +46,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -403,113 +410,167 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+    <col width="12.42578125" customWidth="1" min="1" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>LEN</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>TTAN</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>ULTA</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>445</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="1">
-        <v>108</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1">
-        <v>9</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1">
-        <v>6</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1">
-        <v>12</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated column references for new format
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" customWidth="1" min="1" max="5"/>
@@ -448,131 +448,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>ADBE</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>LEN</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>88</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>TTAN</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>ULTA</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed Schwab_Auth to ask for a full reset each time I run it.  This way I can reset as needed
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" customWidth="1" min="1" max="5"/>
@@ -448,6 +448,31 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>SMTC</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed sheet name in Live_Trade_Info
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,33 +1,70 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading_Algo/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_56BD3A14941E1F658F532FBCD76060A7598B8061" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B480A6B3-AF05-4801-A13F-EEE9C5E58650}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily_Trades" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>Ticker</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Share Size</t>
+  </si>
+  <si>
+    <t>IBKR Exit</t>
+  </si>
+  <si>
+    <t>ToS Exit</t>
+  </si>
+  <si>
+    <t>SMTC</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>MOC</t>
+  </si>
+  <si>
+    <t>long</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,84 +83,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -410,67 +392,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="12.42578125" customWidth="1" min="1" max="5"/>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>SMTC</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1">
         <v>15</v>
       </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a check in Live_Trade_Info to see if I want to trade in single mode, or multi-day mode
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -8,19 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading_Algo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_56BD3A14941E1F658F532FBCD76060A7598B8061" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B480A6B3-AF05-4801-A13F-EEE9C5E58650}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_56BD3A14941E1F658F532FBCD76060A7598B8061" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAD65653-6F88-461F-B9C3-6A0D3F062DE1}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily_Trades" sheetId="1" r:id="rId1"/>
+    <sheet name="Trade_Mode" sheetId="2" r:id="rId1"/>
+    <sheet name="Daily_Trades" sheetId="1" r:id="rId2"/>
+    <sheet name="Monday" sheetId="3" r:id="rId3"/>
+    <sheet name="Tuesday" sheetId="4" r:id="rId4"/>
+    <sheet name="Wednesday" sheetId="5" r:id="rId5"/>
+    <sheet name="Thursday" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="11">
   <si>
     <t>Ticker</t>
   </si>
@@ -47,15 +52,28 @@
   </si>
   <si>
     <t>long</t>
+  </si>
+  <si>
+    <t>Single Day</t>
+  </si>
+  <si>
+    <t>Trade Mode</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,14 +96,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -392,6 +431,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBAB043F-384C-4150-B851-CFCA3E1460A7}">
+  <dimension ref="C2:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -436,4 +499,152 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D685D76F-37FB-41A3-B47E-622C35031175}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9613CE7-597D-4E74-9F59-14106C714343}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ED5B21B-CEBF-49E7-BBD6-571FE038F91B}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2668A4-A61C-40F4-82E2-48EE2853366E}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Created Get_Open_ToS and Get_Closes_ToS in prep os using them
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="3" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="2" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Trade_Mode" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,14 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -54,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999816888943144"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -97,7 +105,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -556,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" customWidth="1" min="1" max="5"/>
@@ -589,12 +597,350 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>STE</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LAR</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>ZBRA</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.42578125" customWidth="1" min="1" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.42578125" customWidth="1" min="1" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>STN</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -636,7 +982,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -645,7 +991,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -655,119 +1001,6 @@
       <c r="E2" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12.42578125" customWidth="1" min="1" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>STZ</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12.42578125" customWidth="1" min="1" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
         </is>
       </c>
     </row>
@@ -818,16 +1051,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -843,7 +1076,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -852,7 +1085,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Made so Exit Order scripts work with latest earnigns doc open
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading_Algo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_D758C3F8449633F930896437798D21188605F9E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B60A92A2-D754-4134-BC1A-6AB071FE01FB}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{DC594C75-2719-4ADD-A16C-7FCF05A9AA30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{197089CF-0F8A-49CA-89B4-94093CA24A14}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Trade_Mode" sheetId="1" r:id="rId1"/>
-    <sheet name="Daily_Trades" sheetId="2" r:id="rId2"/>
+    <sheet name="Daily_Trades" sheetId="1" r:id="rId1"/>
+    <sheet name="Trade_Mode" sheetId="2" r:id="rId2"/>
     <sheet name="Monday" sheetId="3" r:id="rId3"/>
     <sheet name="Tuesday" sheetId="4" r:id="rId4"/>
     <sheet name="Wednesday" sheetId="5" r:id="rId5"/>
@@ -26,7 +26,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="33">
+  <si>
+    <t>Trade Mode</t>
+  </si>
+  <si>
+    <t>Multiday</t>
+  </si>
+  <si>
+    <t>"Single Day", or</t>
+  </si>
+  <si>
+    <t>"Multiday"</t>
+  </si>
   <si>
     <t>Ticker</t>
   </si>
@@ -43,49 +55,76 @@
     <t>ToS Exit</t>
   </si>
   <si>
+    <t>EXP</t>
+  </si>
+  <si>
+    <t>long</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>MOC</t>
+  </si>
+  <si>
+    <t>HD</t>
+  </si>
+  <si>
+    <t>short</t>
+  </si>
+  <si>
+    <t>CAVA</t>
+  </si>
+  <si>
+    <t>TOL</t>
+  </si>
+  <si>
+    <t>ADI</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>TGT</t>
+  </si>
+  <si>
+    <t>TJX</t>
+  </si>
+  <si>
+    <t>WSM</t>
+  </si>
+  <si>
+    <t>ELF</t>
+  </si>
+  <si>
+    <t>INTU</t>
+  </si>
+  <si>
+    <t>NVDA</t>
+  </si>
+  <si>
+    <t>URBN</t>
+  </si>
+  <si>
+    <t>BJ</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>RL</t>
+  </si>
+  <si>
+    <t>WMS</t>
+  </si>
+  <si>
+    <t>WMT</t>
+  </si>
+  <si>
     <t>AMAT</t>
   </si>
   <si>
-    <t>long</t>
-  </si>
-  <si>
-    <t>Open</t>
-  </si>
-  <si>
-    <t>MOC</t>
-  </si>
-  <si>
-    <t>Trade Mode</t>
-  </si>
-  <si>
-    <t>Multiday</t>
-  </si>
-  <si>
-    <t>"Single Day", or</t>
-  </si>
-  <si>
-    <t>"Multiday"</t>
-  </si>
-  <si>
-    <t>EXP</t>
-  </si>
-  <si>
-    <t>HD</t>
-  </si>
-  <si>
-    <t>short</t>
-  </si>
-  <si>
-    <t>CAVA</t>
-  </si>
-  <si>
-    <t>CSCO</t>
-  </si>
-  <si>
-    <t>DOCS</t>
-  </si>
-  <si>
-    <t>STN</t>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -480,6 +519,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
@@ -491,57 +560,27 @@
   <sheetData>
     <row r="2" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C10" s="3" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="5" width="12.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -555,53 +594,53 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -619,79 +658,139 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1">
-        <v>12</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -700,7 +799,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="12.42578125" customWidth="1"/>
@@ -708,70 +807,172 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="1">
+        <v>6</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="1">
+        <v>6</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -789,36 +990,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -836,19 +1037,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Allowed excel to be open for get opens and get closes
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -608,6 +608,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.42578125" customWidth="1" min="1" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -644,16 +688,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -663,50 +707,6 @@
       <c r="E2" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12.42578125" customWidth="1" min="1" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
         </is>
       </c>
     </row>

</xml_diff>